<commit_message>
add PCB design to project
</commit_message>
<xml_diff>
--- a/upload_files/RTM_continuous_config.xlsx
+++ b/upload_files/RTM_continuous_config.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Config"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
   <si>
     <t>Step</t>
   </si>
@@ -57,6 +57,12 @@
   </si>
   <si>
     <t>CW</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>CCW</t>
@@ -103,7 +109,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,12 +127,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -168,6 +168,9 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -183,12 +186,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -495,21 +492,21 @@
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="19.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="58.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>16</v>
+      <c r="A1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
@@ -517,7 +514,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1">
         <v>800</v>
@@ -525,7 +522,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1">
         <v>200</v>
@@ -533,73 +530,73 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="2"/>
-      <c r="B5" s="9"/>
+      <c r="B5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="2"/>
-      <c r="B6" s="9"/>
+      <c r="B6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="9"/>
+      <c r="A7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="9"/>
+        <v>23</v>
+      </c>
+      <c r="B8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="9"/>
+        <v>24</v>
+      </c>
+      <c r="B9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="9"/>
+        <v>25</v>
+      </c>
+      <c r="B10" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="9"/>
+        <v>26</v>
+      </c>
+      <c r="B11" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="9"/>
+        <v>27</v>
+      </c>
+      <c r="B12" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="B13" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="2"/>
-      <c r="B14" s="9"/>
+      <c r="B14" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="2"/>
-      <c r="B15" s="9"/>
+      <c r="B15" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="7"/>
-      <c r="B16" s="9"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="2"/>
-      <c r="B17" s="9"/>
+      <c r="B17" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="2"/>
-      <c r="B18" s="9"/>
+      <c r="B18" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -614,12 +611,12 @@
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="18.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -670,16 +667,16 @@
         <v>12</v>
       </c>
       <c r="C3" s="3">
-        <v>20</v>
+        <v>3000</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="3">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F3" s="3">
-        <v>5</v>
+        <v>72000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -687,440 +684,272 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="3">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="F4" s="3">
-        <v>5</v>
+        <v>14400</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3">
-        <v>60</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="3">
-        <v>350</v>
-      </c>
-      <c r="F5" s="3">
-        <v>5</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="3">
-        <v>350</v>
-      </c>
-      <c r="F6" s="3">
-        <v>5</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="3">
-        <v>40</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="3">
-        <v>350</v>
-      </c>
-      <c r="F7" s="3">
-        <v>5</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="3">
-        <v>60</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="3">
-        <v>350</v>
-      </c>
-      <c r="F8" s="3">
-        <v>5</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="3">
-        <v>20</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="3">
-        <v>350</v>
-      </c>
-      <c r="F9" s="3">
-        <v>5</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="3">
-        <v>40</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="3">
-        <v>350</v>
-      </c>
-      <c r="F10" s="3">
-        <v>5</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="3">
-        <v>60</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="3">
-        <v>350</v>
-      </c>
-      <c r="F11" s="3">
-        <v>5</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="1">
-        <v>10</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="3">
-        <v>300</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="3">
-        <v>350</v>
-      </c>
-      <c r="F12" s="3">
-        <v>5</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="3">
-        <v>800</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="3">
-        <v>500</v>
-      </c>
-      <c r="F13" s="3">
-        <v>11</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="1">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="3">
-        <v>800</v>
-      </c>
-      <c r="F14" s="3">
-        <v>11</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="1">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="3">
-        <v>1000</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="3">
-        <v>500</v>
-      </c>
-      <c r="F15" s="3">
-        <v>2</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="1">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="3">
-        <v>300</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="3">
-        <v>350</v>
-      </c>
-      <c r="F16" s="3">
-        <v>2</v>
-      </c>
+      <c r="A16" s="1"/>
+      <c r="B16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="1">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="3">
-        <v>1000</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="3">
-        <v>350</v>
-      </c>
-      <c r="F17" s="3">
-        <v>2</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="3">
-        <v>300</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="3">
-        <v>350</v>
-      </c>
-      <c r="F18" s="3">
-        <v>2</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="1">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="3">
-        <v>1000</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="3">
-        <v>350</v>
-      </c>
-      <c r="F19" s="3">
-        <v>2</v>
-      </c>
+      <c r="A19" s="1"/>
+      <c r="B19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
-      <c r="A20" s="1">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="3">
-        <v>300</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="3">
-        <v>350</v>
-      </c>
-      <c r="F20" s="3">
-        <v>2</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
-      <c r="A21" s="1">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="3">
-        <v>1000</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="3">
-        <v>350</v>
-      </c>
-      <c r="F21" s="3">
-        <v>2</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="3">
-        <v>300</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="3">
-        <v>350</v>
-      </c>
-      <c r="F22" s="3">
-        <v>2</v>
-      </c>
+      <c r="A22" s="1"/>
+      <c r="B22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" s="3">
-        <v>1000</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="3">
-        <v>350</v>
-      </c>
-      <c r="F23" s="3">
-        <v>2</v>
-      </c>
+      <c r="A23" s="1"/>
+      <c r="B23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="3"/>
+      <c r="D23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="1">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="3">
-        <v>300</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="3">
-        <v>350</v>
-      </c>
-      <c r="F24" s="3">
-        <v>2</v>
-      </c>
+      <c r="A24" s="1"/>
+      <c r="B24" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="1">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="3">
-        <v>800</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="3">
-        <v>500</v>
-      </c>
-      <c r="F25" s="3">
-        <v>11</v>
-      </c>
+      <c r="A25" s="1"/>
+      <c r="B25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="1">
@@ -1133,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E26" s="3">
         <v>800</v>

</xml_diff>

<commit_message>
fixed pre-heating bug and added custom SPR for odd-motor PPR
</commit_message>
<xml_diff>
--- a/upload_files/RTM_continuous_config.xlsx
+++ b/upload_files/RTM_continuous_config.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Step</t>
   </si>
@@ -62,12 +62,6 @@
     <t>false</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>CCW</t>
-  </si>
-  <si>
     <t>Setting</t>
   </si>
   <si>
@@ -81,6 +75,9 @@
   </si>
   <si>
     <t>SPR_3</t>
+  </si>
+  <si>
+    <t>customSPR</t>
   </si>
   <si>
     <t>Note:</t>
@@ -109,7 +106,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,13 +115,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -158,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -169,9 +159,6 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -181,10 +168,10 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -492,89 +479,91 @@
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="58.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="58.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>18</v>
+      <c r="A1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
         <v>200</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2"/>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="B5" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="2"/>
       <c r="B6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="8" t="s">
-        <v>22</v>
+      <c r="A7" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="B7" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1"/>
     </row>
@@ -587,7 +576,7 @@
       <c r="B15" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="8"/>
+      <c r="A16" s="7"/>
       <c r="B16" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
@@ -611,12 +600,12 @@
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="18.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -667,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="3">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>13</v>
@@ -701,275 +690,179 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B5" s="2"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1"/>
-      <c r="B6" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B6" s="2"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1"/>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1"/>
-      <c r="B8" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D8" s="2"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1"/>
-      <c r="B9" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B9" s="2"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D9" s="2"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1"/>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B10" s="2"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1"/>
-      <c r="B11" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B11" s="2"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D11" s="2"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1"/>
-      <c r="B12" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B12" s="2"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D12" s="2"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1"/>
-      <c r="B13" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B13" s="2"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D13" s="2"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1"/>
-      <c r="B14" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B14" s="2"/>
       <c r="C14" s="3"/>
-      <c r="D14" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D14" s="2"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1"/>
-      <c r="B15" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B15" s="2"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D15" s="2"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1"/>
-      <c r="B16" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B16" s="2"/>
       <c r="C16" s="3"/>
-      <c r="D16" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D16" s="2"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1"/>
-      <c r="B17" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B17" s="2"/>
       <c r="C17" s="3"/>
-      <c r="D17" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1"/>
-      <c r="B18" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B18" s="2"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D18" s="2"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1"/>
-      <c r="B19" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B19" s="2"/>
       <c r="C19" s="3"/>
-      <c r="D19" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D19" s="2"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="1"/>
-      <c r="B20" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B20" s="2"/>
       <c r="C20" s="3"/>
-      <c r="D20" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1"/>
-      <c r="B21" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B21" s="2"/>
       <c r="C21" s="3"/>
-      <c r="D21" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D21" s="2"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1"/>
-      <c r="B22" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B22" s="2"/>
       <c r="C22" s="3"/>
-      <c r="D22" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D22" s="2"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1"/>
-      <c r="B23" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B23" s="2"/>
       <c r="C23" s="3"/>
-      <c r="D23" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D23" s="2"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="1"/>
-      <c r="B24" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B24" s="2"/>
       <c r="C24" s="3"/>
-      <c r="D24" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D24" s="2"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="1"/>
-      <c r="B25" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B25" s="2"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="D25" s="2"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="1">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="3">
-        <v>0</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" s="3">
-        <v>800</v>
-      </c>
-      <c r="F26" s="3">
-        <v>11</v>
-      </c>
+      <c r="A26" s="1"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed restart bugs, temp dwell bugs.
</commit_message>
<xml_diff>
--- a/upload_files/RTM_continuous_config.xlsx
+++ b/upload_files/RTM_continuous_config.xlsx
@@ -496,7 +496,7 @@
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -656,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="3">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>13</v>

</xml_diff>